<commit_message>
Expand priority Wordstat coverage
</commit_message>
<xml_diff>
--- a/assets/documents/services-price-current.xlsx
+++ b/assets/documents/services-price-current.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прайс" sheetId="1" r:id="R84860241b9e84257"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прайс" sheetId="1" r:id="R69dfa56b44974f11"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10606,7 +10606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b7c615ba6f94a5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe2c307499394411"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand ultrasound and cosmetology Wordstat data
</commit_message>
<xml_diff>
--- a/assets/documents/services-price-current.xlsx
+++ b/assets/documents/services-price-current.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прайс" sheetId="1" r:id="R69dfa56b44974f11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прайс" sheetId="1" r:id="R1591f04979474253"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10606,7 +10606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe2c307499394411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7566a9d7e8ec4eb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>